<commit_message>
feat: Add Well +a
- 우물 new version 추가
</commit_message>
<xml_diff>
--- a/CSVDatas/InteractivesCSV.xlsx
+++ b/CSVDatas/InteractivesCSV.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PU_Project\_TeamProjects\Retri\_Git\ReTri\CSVDatas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57D95785-066C-4DC5-BB3F-DEF106E64C91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E64625BA-F49E-493F-8238-04CA99C4ED7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="3" xr2:uid="{AFBEF995-9824-4DBC-9BD6-E0A7B4B73573}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="4" xr2:uid="{AFBEF995-9824-4DBC-9BD6-E0A7B4B73573}"/>
   </bookViews>
   <sheets>
     <sheet name="ChaosData" sheetId="1" r:id="rId1"/>
     <sheet name="CurseData" sheetId="2" r:id="rId2"/>
     <sheet name="CurseRewardData" sheetId="3" r:id="rId3"/>
-    <sheet name="Sheet1" sheetId="4" r:id="rId4"/>
+    <sheet name="WellData" sheetId="4" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="90">
   <si>
     <t>ChaosName</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -348,6 +349,19 @@
   <si>
     <t>기억 가속</t>
     <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Dialog</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>내 물건보다 네 목숨값이 싸다는 걸 명심해라.</t>
+  </si>
+  <si>
+    <t>이 던전에서 나대던 놈들이 다 어디로 갔을 것 같나.</t>
+  </si>
+  <si>
+    <t>진열장에 네 머리통이 올라가고 싶지 않으면 얌전히 굴어라.</t>
   </si>
 </sst>
 </file>
@@ -1242,4 +1256,44 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{21E1BD7E-8283-4E2C-8885-CB8E7B30C4AD}">
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>